<commit_message>
Add Redefine Surgery (AI roster 168, viability bins 156)
</commit_message>
<xml_diff>
--- a/viability-bins.xlsx
+++ b/viability-bins.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Companies" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Companies!$A$1:$D$156</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Companies!$A$1:$D$157</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,9 +24,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="350">
-  <si>
-    <t xml:space="preserve">Surgical AI viability bins: backing data for the 'Where the 155 companies land' chart</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="352">
+  <si>
+    <t xml:space="preserve">Surgical AI viability bins: backing data for the 'Where the 156 companies land' chart</t>
   </si>
   <si>
     <t xml:space="preserve">Method: bins are the author's hypotheses about the most probable 2031 outcome, assigned from the master roster (status, funding, notes) combined with public-source research, updated July 28, 2026 after a company-by-company verification pass. Large diversified companies (Intuitive, Medtronic, Stryker, J&amp;J, Olympus, Zeiss, Philips, Brainlab, Accuray, ATEC) are represented as incumbent-platform entries. Bins assess category economics, not team or technology quality; corrections are welcome.</t>
@@ -41,7 +41,7 @@
     <t xml:space="preserve">Companies</t>
   </si>
   <si>
-    <t xml:space="preserve">Share of 155</t>
+    <t xml:space="preserve">Share of 156</t>
   </si>
   <si>
     <t xml:space="preserve">INC</t>
@@ -1074,6 +1074,12 @@
   </si>
   <si>
     <t xml:space="preserve">Chalmers and Sahlgrenska spinout with 5 employees, a 7.5 MSEK pre-seed and Vinnova and Women TechEU grants; Swedish MPA approved the first-in-human study on 22 May 2026 but NCT07630610 (n=6) was still listed NOT_YET_RECRUITING at 1 Sep 2026 and there is no CE mark, so the outcome turns on the trial readout and the next financing; the single-use Navari Landmark marker gives a consumable revenue line that pure-software AR peers lack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redefine Surgery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-seed ($10M, Sep 2026) trackerless computer-vision navigation for orthopedics with one implant partner (Catalyst OrthoScience, shoulder); no FDA clearance, no published accuracy validation and no disclosed payment path, so the outcome turns on a first 510(k) and adoption beyond the founding partner</t>
   </si>
 </sst>
 </file>
@@ -1556,8 +1562,8 @@
         <v>10</v>
       </c>
       <c r="D5" s="8" t="n">
-        <f aca="false">C5/155</f>
-        <v>0.0645161290322581</v>
+        <f aca="false">C5/156</f>
+        <v>0.0641025641025641</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1571,8 +1577,8 @@
         <v>5</v>
       </c>
       <c r="D6" s="8" t="n">
-        <f aca="false">C6/155</f>
-        <v>0.032258064516129</v>
+        <f aca="false">C6/156</f>
+        <v>0.0320512820512821</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1586,8 +1592,8 @@
         <v>9</v>
       </c>
       <c r="D7" s="8" t="n">
-        <f aca="false">C7/155</f>
-        <v>0.0580645161290323</v>
+        <f aca="false">C7/156</f>
+        <v>0.0576923076923077</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1601,8 +1607,8 @@
         <v>35</v>
       </c>
       <c r="D8" s="8" t="n">
-        <f aca="false">C8/155</f>
-        <v>0.225806451612903</v>
+        <f aca="false">C8/156</f>
+        <v>0.224358974358974</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1616,8 +1622,8 @@
         <v>25</v>
       </c>
       <c r="D9" s="8" t="n">
-        <f aca="false">C9/155</f>
-        <v>0.161290322580645</v>
+        <f aca="false">C9/156</f>
+        <v>0.16025641025641</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1631,8 +1637,8 @@
         <v>23</v>
       </c>
       <c r="D10" s="8" t="n">
-        <f aca="false">C10/155</f>
-        <v>0.148387096774194</v>
+        <f aca="false">C10/156</f>
+        <v>0.147435897435897</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1643,11 +1649,11 @@
         <v>19</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D11" s="8" t="n">
-        <f aca="false">C11/155</f>
-        <v>0.245161290322581</v>
+        <f aca="false">C11/156</f>
+        <v>0.25</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1661,8 +1667,8 @@
         <v>10</v>
       </c>
       <c r="D12" s="8" t="n">
-        <f aca="false">C12/155</f>
-        <v>0.0645161290322581</v>
+        <f aca="false">C12/156</f>
+        <v>0.0641025641025641</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1671,7 +1677,7 @@
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="7" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D13" s="8" t="n">
         <v>1</v>
@@ -1693,7 +1699,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D156"/>
+  <dimension ref="A1:D157"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
@@ -3858,7 +3864,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="155" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="7" t="s">
         <v>346</v>
       </c>
@@ -3872,7 +3878,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="7" t="s">
         <v>348</v>
       </c>
@@ -3886,8 +3892,22 @@
         <v>349</v>
       </c>
     </row>
+    <row r="157" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="B157" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C157" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D157" s="6" t="s">
+        <v>351</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D156"/>
+  <autoFilter ref="A1:D157"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>